<commit_message>
Update barley ontology Add percentage threshability trait
</commit_message>
<xml_diff>
--- a/ontology/hordeum-props.xlsx
+++ b/ontology/hordeum-props.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="363">
   <si>
     <t>trait_name</t>
   </si>
@@ -1097,6 +1097,12 @@
   </si>
   <si>
     <t>TRAIT: Sprouting tolerance ::: METHOD: SproutTol Estimation ::: SCALE: 1-9 TOL scale</t>
+  </si>
+  <si>
+    <t>Threshability - %</t>
+  </si>
+  <si>
+    <t>TRAIT: Threshability ::: METHOD: Threshability - Observation ::: SCALE: %</t>
   </si>
 </sst>
 </file>
@@ -1428,7 +1434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H167"/>
+  <dimension ref="A1:H168"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -3412,6 +3418,17 @@
         <v>360</v>
       </c>
     </row>
+    <row r="168" spans="1:7">
+      <c r="A168" t="s">
+        <v>361</v>
+      </c>
+      <c r="B168" t="s">
+        <v>9</v>
+      </c>
+      <c r="G168" t="s">
+        <v>362</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>